<commit_message>
suppression pin-all (#427) 7174292bf4f3486f54165648a1b24098ea6d58df
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-admission-date.xlsx
+++ b/main/ig/StructureDefinition-tddui-admission-date.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-26T12:56:49+00:00</t>
+    <t>2026-02-05T13:38:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -111,7 +111,7 @@
     <t>Base Definition</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/StructureDefinition/Extension|4.0.1</t>
+    <t>http://hl7.org/fhir/StructureDefinition/Extension</t>
   </si>
   <si>
     <t>Abstract</t>

</xml_diff>